<commit_message>
GYLDb.CO STD & PP&E + Excel
</commit_message>
<xml_diff>
--- a/data/cox_xlsx/GYLDb.CO.xlsx
+++ b/data/cox_xlsx/GYLDb.CO.xlsx
@@ -11870,13 +11870,31 @@
       <c r="O66" s="15">
         <v>176.87</v>
       </c>
-      <c r="P66" s="16"/>
-      <c r="Q66" s="16"/>
-      <c r="R66" s="16"/>
-      <c r="S66" s="16"/>
-      <c r="T66" s="16"/>
+      <c r="P66" s="16">
+        <f t="shared" ref="P66:T66" si="1">P67+P71+P76+P81+P86</f>
+        <v>178.08</v>
+      </c>
+      <c r="Q66" s="16">
+        <f t="shared" si="1"/>
+        <v>166.28</v>
+      </c>
+      <c r="R66" s="16">
+        <f t="shared" si="1"/>
+        <v>151.73</v>
+      </c>
+      <c r="S66" s="16">
+        <f t="shared" si="1"/>
+        <v>106.43</v>
+      </c>
+      <c r="T66" s="16">
+        <f t="shared" si="1"/>
+        <v>69.37</v>
+      </c>
       <c r="U66" s="16"/>
-      <c r="V66" s="16"/>
+      <c r="V66" s="16">
+        <f>V67+V71+V76+V81+V86</f>
+        <v>64.51</v>
+      </c>
       <c r="W66" s="16"/>
     </row>
     <row r="67" ht="15.0" customHeight="1">

</xml_diff>